<commit_message>
Started Congestion indicators, included LEHD survey in census bureau queries and processing, slight reorganization of BLS configuration file and functions and scripts...
</commit_message>
<xml_diff>
--- a/Indicator_Gen/Python Code/DOF/config/DOF Configuration File.xlsx
+++ b/Indicator_Gen/Python Code/DOF/config/DOF Configuration File.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\Python Code\DOF\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99725F36-2E95-47B9-A460-9D83C9145D1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4661CFD9-D699-4897-B3EF-E16CD78605EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Indicators" sheetId="39" r:id="rId1"/>
@@ -142,10 +142,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>